<commit_message>
Excel con datos actualizados
</commit_message>
<xml_diff>
--- a/26/Análisis_de_Excels/resultados_optimos.xlsx
+++ b/26/Análisis_de_Excels/resultados_optimos.xlsx
@@ -449,7 +449,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>96184.67393162393</v>
+        <v>90356.89392690809</v>
       </c>
     </row>
     <row r="3">
@@ -459,7 +459,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2084192996.635222</v>
+        <v>1863353787.900699</v>
       </c>
     </row>
     <row r="4">
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.01100015640258789</v>
+        <v>0.01700019836425781</v>
       </c>
     </row>
   </sheetData>
@@ -540,7 +540,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>322.2222222222223</v>
+        <v>365.8511548331908</v>
       </c>
       <c r="D2" t="n">
         <v>2</v>
@@ -558,7 +558,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>149.9999999999999</v>
+        <v>150</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
@@ -576,7 +576,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>247.0085470085471</v>
+        <v>249.7243608022051</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
@@ -612,7 +612,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>303.4188034188034</v>
+        <v>214.2600513259196</v>
       </c>
       <c r="D6" t="n">
         <v>1</v>
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>228.2051282051282</v>
+        <v>182.9255774165954</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
@@ -684,10 +684,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>200</v>
+        <v>374.1317365269462</v>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -720,7 +720,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>185.8974358974359</v>
+        <v>233.5500427715996</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
@@ -755,7 +755,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -807,7 +807,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1925.470149253732</v>
+        <v>5074.888622754494</v>
       </c>
     </row>
     <row r="3">
@@ -823,16 +823,16 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>T02</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>12408.58540630183</v>
+        <v>2240</v>
       </c>
     </row>
     <row r="4">
@@ -843,12 +843,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Base</t>
+          <t>Subbase</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>T12</t>
+          <t>T03</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -857,13 +857,13 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>6672.749999999997</v>
+        <v>2240</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>S02</t>
+          <t>S01</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>T02</t>
+          <t>T05</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -882,23 +882,23 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>3828.632478632479</v>
+        <v>2240</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>S02</t>
+          <t>S01</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Base</t>
+          <t>Subbase</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>T12</t>
+          <t>T06</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -907,13 +907,13 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>2325</v>
+        <v>2240</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>S03</t>
+          <t>S01</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -923,7 +923,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>T07</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -932,23 +932,23 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>5218.160256410254</v>
+        <v>2240</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>S03</t>
+          <t>S01</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Subbase</t>
+          <t>Base</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>T02</t>
+          <t>T09</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -957,13 +957,13 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>15000</v>
+        <v>2240</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>S03</t>
+          <t>S01</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -973,7 +973,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>T06</t>
+          <t>T10</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -982,23 +982,23 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>9995.175000000001</v>
+        <v>2192.75</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>S04</t>
+          <t>S01</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Subbase</t>
+          <t>Base</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>T11</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1007,13 +1007,13 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>14449.19010715653</v>
+        <v>2240</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>S04</t>
+          <t>S02</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1028,17 +1028,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>550.8098928434738</v>
+        <v>1783.251697907904</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>S04</t>
+          <t>S02</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1057,23 +1057,23 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>4769.296153846153</v>
+        <v>799.9999999999887</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>S04</t>
+          <t>S02</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Base</t>
+          <t>Subbase</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>T03</t>
+          <t>T05</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1082,13 +1082,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>12994.425</v>
+        <v>735.8552011740181</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>S05</t>
+          <t>S02</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>T07</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1107,48 +1107,48 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>1920</v>
+        <v>74.09830209209561</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>S05</t>
+          <t>S02</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Base</t>
+          <t>Subbase</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>T12</t>
+          <t>T07</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>1440</v>
+        <v>477.5223912601717</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>S06</t>
+          <t>S02</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Subbase</t>
+          <t>Base</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>T08</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1157,32 +1157,1032 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>1487.179487179487</v>
+        <v>789.1447988259815</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>S02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>T09</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>S02</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>T11</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>735.8552011740068</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>S03</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Subbase</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>T01</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>6003.175942208813</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>S03</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Subbase</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>T01</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>1553.935447868177</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>S03</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Subbase</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>T03</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>451.3432835820896</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>S03</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Subbase</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>T03</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>2908.656716417911</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>S03</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Subbase</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>T04</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>451.3432835820896</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>S03</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Subbase</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>T04</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>2908.656716417911</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>S03</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>T06</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>3275.174999999841</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>S03</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>T10</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>3360</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>S03</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>T12</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>3360</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>S04</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Subbase</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>T01</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>8314.795787787371</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>S04</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Subbase</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>T01</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>2065.93421221263</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>S04</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Subbase</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>T02</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>1106.021308810955</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>S04</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Subbase</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>T04</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>585.6716417910447</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>S04</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Subbase</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>T04</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>3774.328358208955</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>S04</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>T05</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>4360</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>S04</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>T07</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>4274.425</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>S04</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>T12</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>4360</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Subbase</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>T01</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>670.3599999999998</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Subbase</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>T01</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Subbase</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>T02</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>479.9999999999999</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Subbase</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>T03</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Subbase</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>T05</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>6.409345447037016</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Subbase</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>T05</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>39.71000000000004</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Subbase</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>T06</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Subbase</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>T08</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>68.77960959853692</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Subbase</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>T08</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>406.405715613109</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Subbase</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>T09</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>438.695329341317</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Subbase</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>T09</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>41.30467065868299</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>T10</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>479.9999999999999</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>T11</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>T12</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
           <t>S06</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Base</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Subbase</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>T01</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>493.8793656841849</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>S06</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Subbase</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>T02</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>S06</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Subbase</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>T03</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>174.5209764886121</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>S06</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Subbase</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>T04</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>S06</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Subbase</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>T07</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>S06</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>T08</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>S06</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>T10</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>399.9999999999999</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>S06</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
         <is>
           <t>T12</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>M1</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>1200</v>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>400.0000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>